<commit_message>
added pacman() and load packages to app.r
</commit_message>
<xml_diff>
--- a/data-raw/Data_for_R_Shiny.xlsx
+++ b/data-raw/Data_for_R_Shiny.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\Data2\Consumer_Prices_Analysis\202304 CPI Custom Aggregate Calculator\Version 20260608 Posit\CPI-Custom-Aggregate-Calculator\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2389039-E7EB-45AD-A2C7-0A4A2C281400}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56CC60DD-1B2B-40A6-A3EA-8D6E1E300B24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{132A062F-714F-41E8-B5CF-262EE6151935}"/>
   </bookViews>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23254" uniqueCount="6550">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23254" uniqueCount="6552">
   <si>
     <t>Canada</t>
   </si>
@@ -20706,6 +20706,12 @@
 &lt;br&gt;
 &lt;br&gt;
 Les métadonnées sont incorrectes ; il ne faut pas utiliser cette application.</t>
+  </si>
+  <si>
+    <t>Product group</t>
+  </si>
+  <si>
+    <t>Groupe de produits</t>
   </si>
 </sst>
 </file>
@@ -101152,10 +101158,10 @@
         <v>4668</v>
       </c>
       <c r="B21" t="s">
-        <v>4286</v>
+        <v>6550</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>4287</v>
+        <v>6551</v>
       </c>
     </row>
     <row r="22" spans="1:3" s="2" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>